<commit_message>
Added the tasks for this sprint
</commit_message>
<xml_diff>
--- a/Deliverables/Sprint/Soen 341 - agile planning.xlsx
+++ b/Deliverables/Sprint/Soen 341 - agile planning.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\louay\Desktop\LZJCO-SOEN341_Project_W26\Deliverables\Sprint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1621C30-F2D6-402D-9B70-7BC7A7E9990E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F16B26-3507-4305-9967-EDA8DF4FA6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,25 @@
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
     <sheet name="Product Backlog" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="63">
   <si>
     <t>Team LZJCO</t>
   </si>
@@ -176,6 +189,75 @@
 Octavian
 Backend:
 Constance</t>
+  </si>
+  <si>
+    <t>User will be able to see his weekly mean plan</t>
+  </si>
+  <si>
+    <t>User will be able to assign meals to the day of the week and its type (breakfast/lunch/dinner/snack)</t>
+  </si>
+  <si>
+    <t>-Deisng the UI for the weekkly meal plan
+-Have the ability to go to the next/previous week
+-Have the week start at Sunday and end on Saturday
+-Upon clicking on the day of the week, Buttons to add, eidt and remove meals from the day will appear</t>
+  </si>
+  <si>
+    <t>-Upon clicking on the add recipe button for a day, get all recipes from the database and assign it to that day
+-Meals should also get a type that will be assigned to them (breakfast/lunch/dinner/snack)</t>
+  </si>
+  <si>
+    <t>User will be able to edit or remove meals from a day</t>
+  </si>
+  <si>
+    <t>-Upon clicking on the remove/edit button, prompt the user to select which recipe of that day they want to remove/edit
+-Remove/edit that specific meal</t>
+  </si>
+  <si>
+    <t>Frontend: 
+Octavian</t>
+  </si>
+  <si>
+    <t>Constance</t>
+  </si>
+  <si>
+    <t>Cedric</t>
+  </si>
+  <si>
+    <t>HIGH: If there's no way to display recipes in a weekly manner, there is also no way to create/edit/remove recipes</t>
+  </si>
+  <si>
+    <t>System will prevent duplicate meal assignments in the same week</t>
+  </si>
+  <si>
+    <t>-Implement duplicate validation logic
+-Check if recipe already exists in same week
+-Prevent overwrite
+-Display error message</t>
+  </si>
+  <si>
+    <t>System will automatically test  every push and pull request made</t>
+  </si>
+  <si>
+    <t>-Write test cases
+-Validate CRUD operations
+-Test duplicate prevention
+-Perform integration testing</t>
+  </si>
+  <si>
+    <t>HIGH: If there is no recipe added, then it is impossible to edit/remove them</t>
+  </si>
+  <si>
+    <t>MEDIUM: User cannot modify weekly plan</t>
+  </si>
+  <si>
+    <t>Zaree</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> LOW: It does not affect any other task</t>
+  </si>
+  <si>
+    <t>LOW: It does not affect ay other task</t>
   </si>
 </sst>
 </file>
@@ -338,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -387,6 +469,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -613,13 +698,13 @@
     <col min="3" max="3" width="47.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C3" s="1"/>
     </row>
     <row r="4" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -627,10 +712,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C6" s="1"/>
     </row>
     <row r="7" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -638,95 +723,95 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C9" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C10" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C11" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C12" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C13" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C16" s="1"/>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C17" s="1"/>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C19" s="1"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C20" s="1"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C21" s="1"/>
     </row>
-    <row r="22" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C22" s="1"/>
     </row>
-    <row r="23" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C23" s="1"/>
     </row>
-    <row r="24" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C24" s="1"/>
     </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C25" s="1"/>
     </row>
-    <row r="26" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C26" s="1"/>
     </row>
-    <row r="27" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C27" s="1"/>
     </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C28" s="1"/>
     </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C29" s="1"/>
     </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C30" s="1"/>
     </row>
-    <row r="31" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C32" s="1"/>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C35" s="1"/>
     </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C36" s="1"/>
     </row>
     <row r="37" spans="3:3" ht="12.75" x14ac:dyDescent="0.2">
@@ -4078,17 +4163,31 @@
       <c r="Y11" s="5"/>
       <c r="Z11" s="5"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26" ht="157.5" x14ac:dyDescent="0.2">
       <c r="A12" s="10">
         <v>8</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="14"/>
+      <c r="B12" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="12">
+        <v>4</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="14">
+        <v>46099</v>
+      </c>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
@@ -4108,17 +4207,31 @@
       <c r="Y12" s="5"/>
       <c r="Z12" s="5"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" ht="157.5" x14ac:dyDescent="0.2">
       <c r="A13" s="10">
         <v>9</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="14"/>
+      <c r="B13" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="12">
+        <v>6</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H13" s="14">
+        <v>46101</v>
+      </c>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -4138,17 +4251,31 @@
       <c r="Y13" s="5"/>
       <c r="Z13" s="5"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26" ht="110.25" x14ac:dyDescent="0.2">
       <c r="A14" s="10">
         <v>10</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="14"/>
+      <c r="B14" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="12">
+        <v>5</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" s="14">
+        <v>46102</v>
+      </c>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
@@ -4168,17 +4295,31 @@
       <c r="Y14" s="5"/>
       <c r="Z14" s="5"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" ht="94.5" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
         <v>11</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="14"/>
+      <c r="B15" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="12">
+        <v>2</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H15" s="14">
+        <v>46102</v>
+      </c>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -4198,17 +4339,31 @@
       <c r="Y15" s="5"/>
       <c r="Z15" s="5"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26" ht="63" x14ac:dyDescent="0.2">
       <c r="A16" s="10">
         <v>12</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="14"/>
+      <c r="B16" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="12">
+        <v>5</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H16" s="14">
+        <v>46102</v>
+      </c>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>

</xml_diff>

<commit_message>
Added individual story points per sprint
</commit_message>
<xml_diff>
--- a/Deliverables/Sprint/Soen 341 - agile planning.xlsx
+++ b/Deliverables/Sprint/Soen 341 - agile planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\louay\Desktop\LZJCO-SOEN341_Project_W26\Deliverables\Sprint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0A9A62-5C46-4D6F-826D-0454E23F56F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8DE2B6C-0231-47BE-B989-17911A11535F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="82">
   <si>
     <t>Team LZJCO</t>
   </si>
@@ -311,6 +311,24 @@
     <t>-Write unit test for all code
 -write at least 2 acceptance tests for all user stories</t>
   </si>
+  <si>
+    <t>Sprint 1</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <t>Octav</t>
+  </si>
+  <si>
+    <t>Story Points per sprint</t>
+  </si>
 </sst>
 </file>
 
@@ -538,7 +556,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -642,6 +660,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4149,7 +4173,10 @@
       <c r="A7" s="14"/>
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
+      <c r="D7" s="15">
+        <f>SUM(D3:D6)</f>
+        <v>17</v>
+      </c>
       <c r="E7" s="15"/>
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
@@ -4309,7 +4336,10 @@
       <c r="A11" s="14"/>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
-      <c r="D11" s="15"/>
+      <c r="D11" s="15">
+        <f>SUM(D8:D10)</f>
+        <v>15</v>
+      </c>
       <c r="E11" s="15"/>
       <c r="F11" s="15"/>
       <c r="G11" s="15"/>
@@ -4476,7 +4506,7 @@
         <v>67</v>
       </c>
       <c r="D15" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>29</v>
@@ -4564,7 +4594,7 @@
         <v>63</v>
       </c>
       <c r="D17" s="11">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>29</v>
@@ -4691,7 +4721,10 @@
       </c>
       <c r="B20" s="29"/>
       <c r="C20" s="33"/>
-      <c r="D20" s="29"/>
+      <c r="D20" s="29">
+        <f>SUM(D12:D19)</f>
+        <v>33</v>
+      </c>
       <c r="E20" s="29"/>
       <c r="F20" s="29"/>
       <c r="G20" s="29"/>
@@ -4896,12 +4929,14 @@
       <c r="F26" s="31"/>
       <c r="G26" s="31"/>
       <c r="H26" s="31"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
+      <c r="I26" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="J26" s="37"/>
+      <c r="K26" s="37"/>
+      <c r="L26" s="37"/>
+      <c r="M26" s="37"/>
+      <c r="N26" s="37"/>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
@@ -4924,12 +4959,20 @@
       <c r="F27" s="31"/>
       <c r="G27" s="31"/>
       <c r="H27" s="31"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-      <c r="M27" s="4"/>
-      <c r="N27" s="4"/>
+      <c r="I27" s="36"/>
+      <c r="J27" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="K27" s="36" t="s">
+        <v>77</v>
+      </c>
+      <c r="L27" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="M27" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="N27" s="36"/>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
@@ -4952,12 +4995,25 @@
       <c r="F28" s="31"/>
       <c r="G28" s="31"/>
       <c r="H28" s="31"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
-      <c r="M28" s="4"/>
-      <c r="N28" s="4"/>
+      <c r="I28" s="36" t="s">
+        <v>64</v>
+      </c>
+      <c r="J28" s="36">
+        <v>4</v>
+      </c>
+      <c r="K28" s="36">
+        <v>3</v>
+      </c>
+      <c r="L28" s="36">
+        <v>8</v>
+      </c>
+      <c r="M28" s="36">
+        <v>1</v>
+      </c>
+      <c r="N28" s="36">
+        <f>SUM(J28:M28)</f>
+        <v>16</v>
+      </c>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
@@ -4980,12 +5036,25 @@
       <c r="F29" s="31"/>
       <c r="G29" s="31"/>
       <c r="H29" s="31"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="4"/>
-      <c r="M29" s="4"/>
-      <c r="N29" s="4"/>
+      <c r="I29" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="J29" s="36">
+        <v>3</v>
+      </c>
+      <c r="K29" s="36">
+        <v>3</v>
+      </c>
+      <c r="L29" s="36">
+        <v>7</v>
+      </c>
+      <c r="M29" s="36">
+        <v>1</v>
+      </c>
+      <c r="N29" s="36">
+        <f t="shared" ref="N29:N32" si="0">SUM(J29:M29)</f>
+        <v>14</v>
+      </c>
       <c r="O29" s="4"/>
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
@@ -5008,12 +5077,25 @@
       <c r="F30" s="31"/>
       <c r="G30" s="31"/>
       <c r="H30" s="31"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
+      <c r="I30" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="J30" s="36">
+        <v>4</v>
+      </c>
+      <c r="K30" s="36">
+        <v>3</v>
+      </c>
+      <c r="L30" s="36">
+        <v>6</v>
+      </c>
+      <c r="M30" s="36">
+        <v>1</v>
+      </c>
+      <c r="N30" s="36">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
@@ -5036,12 +5118,25 @@
       <c r="F31" s="31"/>
       <c r="G31" s="31"/>
       <c r="H31" s="31"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
-      <c r="M31" s="4"/>
-      <c r="N31" s="4"/>
+      <c r="I31" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="J31" s="36">
+        <v>3</v>
+      </c>
+      <c r="K31" s="36">
+        <v>3</v>
+      </c>
+      <c r="L31" s="36">
+        <v>7</v>
+      </c>
+      <c r="M31" s="36">
+        <v>1</v>
+      </c>
+      <c r="N31" s="36">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
@@ -5064,12 +5159,25 @@
       <c r="F32" s="31"/>
       <c r="G32" s="31"/>
       <c r="H32" s="31"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
-      <c r="M32" s="4"/>
-      <c r="N32" s="4"/>
+      <c r="I32" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="J32" s="36">
+        <v>3</v>
+      </c>
+      <c r="K32" s="36">
+        <v>3</v>
+      </c>
+      <c r="L32" s="36">
+        <v>5</v>
+      </c>
+      <c r="M32" s="36">
+        <v>5</v>
+      </c>
+      <c r="N32" s="36">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
@@ -5092,12 +5200,24 @@
       <c r="F33" s="31"/>
       <c r="G33" s="31"/>
       <c r="H33" s="31"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4"/>
+      <c r="I33" s="36"/>
+      <c r="J33" s="36">
+        <f>SUM(J28:J32)</f>
+        <v>17</v>
+      </c>
+      <c r="K33" s="36">
+        <f t="shared" ref="K33:M33" si="1">SUM(K28:K32)</f>
+        <v>15</v>
+      </c>
+      <c r="L33" s="36">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+      <c r="M33" s="36">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="N33" s="36"/>
       <c r="O33" s="4"/>
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
@@ -31992,6 +32112,9 @@
       <c r="Z993" s="5"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I26:N26"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="597" r:id="rId1"/>
 </worksheet>

</xml_diff>